<commit_message>
autres modofs + spectre solaire
</commit_message>
<xml_diff>
--- a/Projet_1/Projet 1.xlsx
+++ b/Projet_1/Projet 1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29910"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/e8cc6f8fcd8ecae5/Bureau/Labos-TPOP/Projet_1/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\alext\OneDrive\Bureau\Génie physique\Calculs python\Labos-TPOP\Projet_1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="389" documentId="13_ncr:1_{38C6B4CF-A780-477D-A32A-F81D924AC5EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B0DC38E0-CBA1-4180-B69A-5649E0AAA0D0}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5B8F7E5-3E26-4CE5-87D7-C8B0EC35DC6A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="9585" yWindow="1950" windowWidth="14400" windowHeight="8175" firstSheet="2" activeTab="4" xr2:uid="{09CE5A8B-92B7-4C41-A704-2A22CC0EC3FE}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" firstSheet="2" activeTab="5" xr2:uid="{09CE5A8B-92B7-4C41-A704-2A22CC0EC3FE}"/>
   </bookViews>
   <sheets>
     <sheet name="Code python" sheetId="1" r:id="rId1"/>
@@ -18,6 +18,7 @@
     <sheet name="Obj2" sheetId="3" r:id="rId3"/>
     <sheet name="Obj3" sheetId="4" r:id="rId4"/>
     <sheet name="Obj4" sheetId="5" r:id="rId5"/>
+    <sheet name="Spectre" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -40,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="24">
   <si>
     <t>Code python</t>
   </si>
@@ -92,18 +93,56 @@
   <si>
     <t>Temps (minutes)</t>
   </si>
+  <si>
+    <t>Wavelength</t>
+  </si>
+  <si>
+    <t>Spectral irradiance</t>
+  </si>
+  <si>
+    <t>Cumulative photon flux</t>
+  </si>
+  <si>
+    <t>Wavelength (nm)</t>
+  </si>
+  <si>
+    <t>Spectral irradiance (W⋅m–2⋅nm–1)</t>
+  </si>
+  <si>
+    <t>Cumulative photon flux (cm–2⋅s–1)</t>
+  </si>
+  <si>
+    <t>https://www2.pvlighthouse.com.au/resources/optics/spectrum%20library/spectrum%20library.aspx</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <name val="Verdana"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Verdana"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -120,7 +159,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="18">
+  <borders count="19">
     <border>
       <left/>
       <right/>
@@ -313,11 +352,20 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FF193C3C"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -397,8 +445,18 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="11" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -420,7 +478,7 @@
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="fr-FR"/>
+  <c:lang val="en-US"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -1944,7 +2002,7 @@
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="fr-FR"/>
+  <c:lang val="en-US"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -4226,9 +4284,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7D2746A0-2681-4FDC-B6E1-17CB27A8811C}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="14.45"/>
+  <sheetFormatPr defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:1">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -4241,17 +4299,17 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{061E08D7-867C-40CF-B00D-4C3BCEF18156}">
   <dimension ref="A3:A5"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="14.45"/>
+  <sheetFormatPr defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="22.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="22.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:1">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:1">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>2</v>
       </c>
@@ -4264,13 +4322,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{61BB71E7-EDC9-4678-B0D6-C45A85E23791}">
   <dimension ref="A2:G46"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="8.7265625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="9" width="16.42578125" style="2" customWidth="1"/>
-    <col min="10" max="16384" width="8.7109375" style="2"/>
+    <col min="1" max="9" width="16.453125" style="2" customWidth="1"/>
+    <col min="10" max="16384" width="8.7265625" style="2"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:7" s="1" customFormat="1">
+    <row r="2" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A2" s="6" t="s">
         <v>3</v>
       </c>
@@ -4291,11 +4349,11 @@
       </c>
       <c r="G2" s="8"/>
     </row>
-    <row r="3" spans="1:7">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" s="3">
         <v>0</v>
       </c>
-      <c r="B3" s="33">
+      <c r="B3" s="2">
         <f>A3*2.54</f>
         <v>0</v>
       </c>
@@ -4313,11 +4371,11 @@
       </c>
       <c r="G3" s="4"/>
     </row>
-    <row r="4" spans="1:7">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4" s="3">
         <v>1</v>
       </c>
-      <c r="B4" s="33">
+      <c r="B4" s="2">
         <f t="shared" ref="B4:B46" si="0">A4*2.54</f>
         <v>2.54</v>
       </c>
@@ -4335,11 +4393,11 @@
       </c>
       <c r="G4" s="4"/>
     </row>
-    <row r="5" spans="1:7">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5" s="3">
         <v>2</v>
       </c>
-      <c r="B5" s="33">
+      <c r="B5" s="2">
         <f t="shared" si="0"/>
         <v>5.08</v>
       </c>
@@ -4357,11 +4415,11 @@
       </c>
       <c r="G5" s="4"/>
     </row>
-    <row r="6" spans="1:7">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A6" s="3">
         <v>3</v>
       </c>
-      <c r="B6" s="33">
+      <c r="B6" s="2">
         <f t="shared" si="0"/>
         <v>7.62</v>
       </c>
@@ -4379,11 +4437,11 @@
       </c>
       <c r="G6" s="4"/>
     </row>
-    <row r="7" spans="1:7">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A7" s="3">
         <v>4</v>
       </c>
-      <c r="B7" s="33">
+      <c r="B7" s="2">
         <f t="shared" si="0"/>
         <v>10.16</v>
       </c>
@@ -4401,11 +4459,11 @@
       </c>
       <c r="G7" s="4"/>
     </row>
-    <row r="8" spans="1:7">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A8" s="3">
         <v>5</v>
       </c>
-      <c r="B8" s="33">
+      <c r="B8" s="2">
         <f t="shared" si="0"/>
         <v>12.7</v>
       </c>
@@ -4423,11 +4481,11 @@
       </c>
       <c r="G8" s="4"/>
     </row>
-    <row r="9" spans="1:7">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A9" s="3">
         <v>6</v>
       </c>
-      <c r="B9" s="33">
+      <c r="B9" s="2">
         <f t="shared" si="0"/>
         <v>15.24</v>
       </c>
@@ -4445,11 +4503,11 @@
       </c>
       <c r="G9" s="4"/>
     </row>
-    <row r="10" spans="1:7">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A10" s="3">
         <v>7</v>
       </c>
-      <c r="B10" s="33">
+      <c r="B10" s="2">
         <f t="shared" si="0"/>
         <v>17.78</v>
       </c>
@@ -4467,11 +4525,11 @@
       </c>
       <c r="G10" s="4"/>
     </row>
-    <row r="11" spans="1:7">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A11" s="3">
         <v>8</v>
       </c>
-      <c r="B11" s="33">
+      <c r="B11" s="2">
         <f t="shared" si="0"/>
         <v>20.32</v>
       </c>
@@ -4489,11 +4547,11 @@
       </c>
       <c r="G11" s="4"/>
     </row>
-    <row r="12" spans="1:7">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A12" s="3">
         <v>9</v>
       </c>
-      <c r="B12" s="33">
+      <c r="B12" s="2">
         <f t="shared" si="0"/>
         <v>22.86</v>
       </c>
@@ -4511,11 +4569,11 @@
       </c>
       <c r="G12" s="12"/>
     </row>
-    <row r="13" spans="1:7">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A13" s="3">
         <v>10</v>
       </c>
-      <c r="B13" s="33">
+      <c r="B13" s="2">
         <f t="shared" si="0"/>
         <v>25.4</v>
       </c>
@@ -4533,11 +4591,11 @@
       </c>
       <c r="G13" s="12"/>
     </row>
-    <row r="14" spans="1:7">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A14" s="3">
         <v>11</v>
       </c>
-      <c r="B14" s="33">
+      <c r="B14" s="2">
         <f t="shared" si="0"/>
         <v>27.94</v>
       </c>
@@ -4555,11 +4613,11 @@
       </c>
       <c r="G14" s="12"/>
     </row>
-    <row r="15" spans="1:7">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A15" s="3">
         <v>12</v>
       </c>
-      <c r="B15" s="33">
+      <c r="B15" s="2">
         <f t="shared" si="0"/>
         <v>30.48</v>
       </c>
@@ -4577,11 +4635,11 @@
       </c>
       <c r="G15" s="12"/>
     </row>
-    <row r="16" spans="1:7">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A16" s="3">
         <v>13</v>
       </c>
-      <c r="B16" s="33">
+      <c r="B16" s="2">
         <f t="shared" si="0"/>
         <v>33.020000000000003</v>
       </c>
@@ -4599,11 +4657,11 @@
       </c>
       <c r="G16" s="12"/>
     </row>
-    <row r="17" spans="1:7">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A17" s="3">
         <v>14</v>
       </c>
-      <c r="B17" s="33">
+      <c r="B17" s="2">
         <f t="shared" si="0"/>
         <v>35.56</v>
       </c>
@@ -4621,11 +4679,11 @@
       </c>
       <c r="G17" s="12"/>
     </row>
-    <row r="18" spans="1:7">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A18" s="3">
         <v>15</v>
       </c>
-      <c r="B18" s="33">
+      <c r="B18" s="2">
         <f t="shared" si="0"/>
         <v>38.1</v>
       </c>
@@ -4643,11 +4701,11 @@
       </c>
       <c r="G18" s="12"/>
     </row>
-    <row r="19" spans="1:7">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A19" s="3">
         <v>16</v>
       </c>
-      <c r="B19" s="33">
+      <c r="B19" s="2">
         <f t="shared" si="0"/>
         <v>40.64</v>
       </c>
@@ -4665,11 +4723,11 @@
       </c>
       <c r="G19" s="25"/>
     </row>
-    <row r="20" spans="1:7">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A20" s="3">
         <v>17</v>
       </c>
-      <c r="B20" s="33">
+      <c r="B20" s="2">
         <f t="shared" si="0"/>
         <v>43.18</v>
       </c>
@@ -4687,11 +4745,11 @@
       </c>
       <c r="G20" s="18"/>
     </row>
-    <row r="21" spans="1:7">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A21" s="3">
         <v>18</v>
       </c>
-      <c r="B21" s="33">
+      <c r="B21" s="2">
         <f t="shared" si="0"/>
         <v>45.72</v>
       </c>
@@ -4709,11 +4767,11 @@
       </c>
       <c r="G21" s="18"/>
     </row>
-    <row r="22" spans="1:7">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A22" s="3">
         <v>19</v>
       </c>
-      <c r="B22" s="33">
+      <c r="B22" s="2">
         <f t="shared" si="0"/>
         <v>48.26</v>
       </c>
@@ -4731,11 +4789,11 @@
       </c>
       <c r="G22" s="18"/>
     </row>
-    <row r="23" spans="1:7">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A23" s="3">
         <v>20</v>
       </c>
-      <c r="B23" s="33">
+      <c r="B23" s="2">
         <f t="shared" si="0"/>
         <v>50.8</v>
       </c>
@@ -4753,11 +4811,11 @@
       </c>
       <c r="G23" s="21"/>
     </row>
-    <row r="24" spans="1:7">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A24" s="3">
         <v>21</v>
       </c>
-      <c r="B24" s="33">
+      <c r="B24" s="2">
         <f t="shared" si="0"/>
         <v>53.34</v>
       </c>
@@ -4774,11 +4832,11 @@
         <v>1081</v>
       </c>
     </row>
-    <row r="25" spans="1:7">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A25" s="3">
         <v>22</v>
       </c>
-      <c r="B25" s="33">
+      <c r="B25" s="2">
         <f t="shared" si="0"/>
         <v>55.88</v>
       </c>
@@ -4795,11 +4853,11 @@
         <v>994</v>
       </c>
     </row>
-    <row r="26" spans="1:7">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A26" s="3">
         <v>23</v>
       </c>
-      <c r="B26" s="33">
+      <c r="B26" s="2">
         <f t="shared" si="0"/>
         <v>58.42</v>
       </c>
@@ -4816,11 +4874,11 @@
         <v>918</v>
       </c>
     </row>
-    <row r="27" spans="1:7">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A27" s="3">
         <v>24</v>
       </c>
-      <c r="B27" s="33">
+      <c r="B27" s="2">
         <f t="shared" si="0"/>
         <v>60.96</v>
       </c>
@@ -4837,11 +4895,11 @@
         <v>851</v>
       </c>
     </row>
-    <row r="28" spans="1:7">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A28" s="3">
         <v>25</v>
       </c>
-      <c r="B28" s="33">
+      <c r="B28" s="2">
         <f t="shared" si="0"/>
         <v>63.5</v>
       </c>
@@ -4858,11 +4916,11 @@
         <v>792</v>
       </c>
     </row>
-    <row r="29" spans="1:7">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A29" s="3">
         <v>26</v>
       </c>
-      <c r="B29" s="33">
+      <c r="B29" s="2">
         <f t="shared" si="0"/>
         <v>66.040000000000006</v>
       </c>
@@ -4879,11 +4937,11 @@
         <v>741</v>
       </c>
     </row>
-    <row r="30" spans="1:7">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A30" s="3">
         <v>27</v>
       </c>
-      <c r="B30" s="33">
+      <c r="B30" s="2">
         <f t="shared" si="0"/>
         <v>68.58</v>
       </c>
@@ -4900,11 +4958,11 @@
         <v>694</v>
       </c>
     </row>
-    <row r="31" spans="1:7">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A31" s="3">
         <v>28</v>
       </c>
-      <c r="B31" s="33">
+      <c r="B31" s="2">
         <f t="shared" si="0"/>
         <v>71.12</v>
       </c>
@@ -4921,11 +4979,11 @@
         <v>651</v>
       </c>
     </row>
-    <row r="32" spans="1:7">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A32" s="3">
         <v>29</v>
       </c>
-      <c r="B32" s="33">
+      <c r="B32" s="2">
         <f t="shared" si="0"/>
         <v>73.66</v>
       </c>
@@ -4942,11 +5000,11 @@
         <v>612</v>
       </c>
     </row>
-    <row r="33" spans="1:6">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A33" s="3">
         <v>30</v>
       </c>
-      <c r="B33" s="33">
+      <c r="B33" s="2">
         <f t="shared" si="0"/>
         <v>76.2</v>
       </c>
@@ -4963,11 +5021,11 @@
         <v>578</v>
       </c>
     </row>
-    <row r="34" spans="1:6">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A34" s="3">
         <v>31</v>
       </c>
-      <c r="B34" s="33">
+      <c r="B34" s="2">
         <f t="shared" si="0"/>
         <v>78.739999999999995</v>
       </c>
@@ -4984,11 +5042,11 @@
         <v>544</v>
       </c>
     </row>
-    <row r="35" spans="1:6">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A35" s="3">
         <v>32</v>
       </c>
-      <c r="B35" s="33">
+      <c r="B35" s="2">
         <f t="shared" si="0"/>
         <v>81.28</v>
       </c>
@@ -5005,11 +5063,11 @@
         <v>514</v>
       </c>
     </row>
-    <row r="36" spans="1:6">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A36" s="3">
         <v>33</v>
       </c>
-      <c r="B36" s="33">
+      <c r="B36" s="2">
         <f t="shared" si="0"/>
         <v>83.820000000000007</v>
       </c>
@@ -5026,11 +5084,11 @@
         <v>488</v>
       </c>
     </row>
-    <row r="37" spans="1:6">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A37" s="3">
         <v>34</v>
       </c>
-      <c r="B37" s="33">
+      <c r="B37" s="2">
         <f t="shared" si="0"/>
         <v>86.36</v>
       </c>
@@ -5047,11 +5105,11 @@
         <v>465</v>
       </c>
     </row>
-    <row r="38" spans="1:6">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A38" s="3">
         <v>35</v>
       </c>
-      <c r="B38" s="33">
+      <c r="B38" s="2">
         <f t="shared" si="0"/>
         <v>88.9</v>
       </c>
@@ -5068,11 +5126,11 @@
         <v>442</v>
       </c>
     </row>
-    <row r="39" spans="1:6">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A39" s="3">
         <v>36</v>
       </c>
-      <c r="B39" s="33">
+      <c r="B39" s="2">
         <f t="shared" si="0"/>
         <v>91.44</v>
       </c>
@@ -5089,11 +5147,11 @@
         <v>422</v>
       </c>
     </row>
-    <row r="40" spans="1:6">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A40" s="3">
         <v>37</v>
       </c>
-      <c r="B40" s="33">
+      <c r="B40" s="2">
         <f t="shared" si="0"/>
         <v>93.98</v>
       </c>
@@ -5110,11 +5168,11 @@
         <v>404</v>
       </c>
     </row>
-    <row r="41" spans="1:6">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A41" s="3">
         <v>38</v>
       </c>
-      <c r="B41" s="33">
+      <c r="B41" s="2">
         <f t="shared" si="0"/>
         <v>96.52</v>
       </c>
@@ -5131,11 +5189,11 @@
         <v>385</v>
       </c>
     </row>
-    <row r="42" spans="1:6">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A42" s="3">
         <v>39</v>
       </c>
-      <c r="B42" s="33">
+      <c r="B42" s="2">
         <f t="shared" si="0"/>
         <v>99.06</v>
       </c>
@@ -5152,11 +5210,11 @@
         <v>367</v>
       </c>
     </row>
-    <row r="43" spans="1:6">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A43" s="3">
         <v>40</v>
       </c>
-      <c r="B43" s="33">
+      <c r="B43" s="2">
         <f t="shared" si="0"/>
         <v>101.6</v>
       </c>
@@ -5173,11 +5231,11 @@
         <v>351</v>
       </c>
     </row>
-    <row r="44" spans="1:6">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A44" s="3">
         <v>41</v>
       </c>
-      <c r="B44" s="33">
+      <c r="B44" s="2">
         <f t="shared" si="0"/>
         <v>104.14</v>
       </c>
@@ -5194,11 +5252,11 @@
         <v>337</v>
       </c>
     </row>
-    <row r="45" spans="1:6">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A45" s="3">
         <v>42</v>
       </c>
-      <c r="B45" s="33">
+      <c r="B45" s="2">
         <f t="shared" si="0"/>
         <v>106.68</v>
       </c>
@@ -5215,11 +5273,11 @@
         <v>323</v>
       </c>
     </row>
-    <row r="46" spans="1:6">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A46" s="3">
         <v>43</v>
       </c>
-      <c r="B46" s="33">
+      <c r="B46" s="2">
         <f t="shared" si="0"/>
         <v>109.22</v>
       </c>
@@ -5245,19 +5303,19 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{077AC35B-C91C-41A7-9EEE-2FE26DB8404D}">
   <dimension ref="A1:G19"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="14.45"/>
+  <sheetFormatPr defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="14.140625" style="9" customWidth="1"/>
-    <col min="2" max="8" width="16.42578125" customWidth="1"/>
+    <col min="1" max="1" width="14.1796875" style="9" customWidth="1"/>
+    <col min="2" max="8" width="16.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
       <c r="D1" s="2"/>
       <c r="G1" s="2"/>
     </row>
-    <row r="2" spans="1:7" ht="44.1" thickBot="1">
+    <row r="2" spans="1:7" ht="44" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A2" s="16" t="s">
         <v>9</v>
       </c>
@@ -5280,7 +5338,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="15" thickTop="1">
+    <row r="3" spans="1:7" ht="15" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A3" s="10"/>
       <c r="B3" s="11">
         <v>-80</v>
@@ -5289,7 +5347,7 @@
       <c r="D3" s="2"/>
       <c r="G3" s="4"/>
     </row>
-    <row r="4" spans="1:7">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4" s="10"/>
       <c r="B4" s="11">
         <v>-70</v>
@@ -5298,7 +5356,7 @@
       <c r="D4" s="2"/>
       <c r="G4" s="4"/>
     </row>
-    <row r="5" spans="1:7">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5" s="10"/>
       <c r="B5" s="11">
         <v>-60</v>
@@ -5307,7 +5365,7 @@
       <c r="D5" s="2"/>
       <c r="G5" s="4"/>
     </row>
-    <row r="6" spans="1:7">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A6" s="10"/>
       <c r="B6" s="11">
         <v>-50</v>
@@ -5316,7 +5374,7 @@
       <c r="D6" s="2"/>
       <c r="G6" s="4"/>
     </row>
-    <row r="7" spans="1:7">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A7" s="10"/>
       <c r="B7" s="11">
         <v>-40</v>
@@ -5325,7 +5383,7 @@
       <c r="D7" s="2"/>
       <c r="G7" s="4"/>
     </row>
-    <row r="8" spans="1:7">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A8" s="10"/>
       <c r="B8" s="11">
         <v>-30</v>
@@ -5334,7 +5392,7 @@
       <c r="D8" s="2"/>
       <c r="G8" s="4"/>
     </row>
-    <row r="9" spans="1:7">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A9" s="10"/>
       <c r="B9" s="11">
         <v>-20</v>
@@ -5343,7 +5401,7 @@
       <c r="D9" s="2"/>
       <c r="G9" s="4"/>
     </row>
-    <row r="10" spans="1:7">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A10" s="10"/>
       <c r="B10" s="11">
         <v>-10</v>
@@ -5352,7 +5410,7 @@
       <c r="D10" s="2"/>
       <c r="G10" s="4"/>
     </row>
-    <row r="11" spans="1:7">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A11" s="10"/>
       <c r="B11" s="2">
         <v>0</v>
@@ -5361,56 +5419,56 @@
       <c r="D11" s="2"/>
       <c r="G11" s="4"/>
     </row>
-    <row r="12" spans="1:7">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A12" s="10"/>
       <c r="B12" s="2">
         <v>10</v>
       </c>
       <c r="G12" s="12"/>
     </row>
-    <row r="13" spans="1:7">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A13" s="10"/>
       <c r="B13" s="2">
         <v>20</v>
       </c>
       <c r="G13" s="12"/>
     </row>
-    <row r="14" spans="1:7">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A14" s="10"/>
       <c r="B14" s="2">
         <v>30</v>
       </c>
       <c r="G14" s="12"/>
     </row>
-    <row r="15" spans="1:7">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A15" s="10"/>
       <c r="B15" s="2">
         <v>40</v>
       </c>
       <c r="G15" s="12"/>
     </row>
-    <row r="16" spans="1:7">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A16" s="10"/>
       <c r="B16" s="2">
         <v>50</v>
       </c>
       <c r="G16" s="12"/>
     </row>
-    <row r="17" spans="1:7">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A17" s="10"/>
       <c r="B17" s="2">
         <v>60</v>
       </c>
       <c r="G17" s="12"/>
     </row>
-    <row r="18" spans="1:7">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A18" s="10"/>
       <c r="B18" s="2">
         <v>70</v>
       </c>
       <c r="G18" s="12"/>
     </row>
-    <row r="19" spans="1:7">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A19" s="13"/>
       <c r="B19" s="5">
         <v>80</v>
@@ -5429,19 +5487,19 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{73B07D6C-4435-41CC-9699-27F599DBF5B1}">
   <dimension ref="A1:F19"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="8" width="16.42578125" customWidth="1"/>
+    <col min="1" max="8" width="16.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" s="2"/>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
       <c r="D1" s="2"/>
       <c r="E1" s="2"/>
     </row>
-    <row r="2" spans="1:6">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2" s="22" t="s">
         <v>3</v>
       </c>
@@ -5461,7 +5519,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:6">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3" s="17">
         <v>5</v>
       </c>
@@ -5481,7 +5539,7 @@
         <v>6320</v>
       </c>
     </row>
-    <row r="4" spans="1:6">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" s="17"/>
       <c r="B4" s="18">
         <v>5</v>
@@ -5499,7 +5557,7 @@
         <v>8460</v>
       </c>
     </row>
-    <row r="5" spans="1:6">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5" s="17"/>
       <c r="B5" s="18">
         <v>10</v>
@@ -5517,7 +5575,7 @@
         <v>6430</v>
       </c>
     </row>
-    <row r="6" spans="1:6">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6" s="17"/>
       <c r="B6" s="18">
         <v>15</v>
@@ -5535,7 +5593,7 @@
         <v>6280</v>
       </c>
     </row>
-    <row r="7" spans="1:6">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7" s="17"/>
       <c r="B7" s="18">
         <v>20</v>
@@ -5553,7 +5611,7 @@
         <v>5900</v>
       </c>
     </row>
-    <row r="8" spans="1:6">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A8" s="17"/>
       <c r="B8" s="18">
         <v>25</v>
@@ -5571,7 +5629,7 @@
         <v>6010</v>
       </c>
     </row>
-    <row r="9" spans="1:6">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A9" s="17"/>
       <c r="B9" s="18">
         <v>30</v>
@@ -5589,7 +5647,7 @@
         <v>6420</v>
       </c>
     </row>
-    <row r="10" spans="1:6">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A10" s="17"/>
       <c r="B10" s="18">
         <v>35</v>
@@ -5607,7 +5665,7 @@
         <v>6140</v>
       </c>
     </row>
-    <row r="11" spans="1:6">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A11" s="17"/>
       <c r="B11" s="18">
         <v>40</v>
@@ -5625,7 +5683,7 @@
         <v>5970</v>
       </c>
     </row>
-    <row r="12" spans="1:6">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A12" s="19"/>
       <c r="B12" s="18">
         <v>45</v>
@@ -5643,7 +5701,7 @@
         <v>6000</v>
       </c>
     </row>
-    <row r="13" spans="1:6">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A13" s="19"/>
       <c r="B13" s="18">
         <v>50</v>
@@ -5661,7 +5719,7 @@
         <v>5990</v>
       </c>
     </row>
-    <row r="14" spans="1:6">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A14" s="19"/>
       <c r="B14" s="18">
         <v>55</v>
@@ -5679,7 +5737,7 @@
         <v>6300</v>
       </c>
     </row>
-    <row r="15" spans="1:6">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A15" s="19"/>
       <c r="B15" s="18">
         <v>60</v>
@@ -5697,28 +5755,28 @@
         <v>6190</v>
       </c>
     </row>
-    <row r="16" spans="1:6">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A16" s="19"/>
       <c r="B16" s="18">
         <v>65</v>
       </c>
       <c r="F16" s="25"/>
     </row>
-    <row r="17" spans="1:6">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A17" s="19"/>
       <c r="B17" s="18">
         <v>70</v>
       </c>
       <c r="F17" s="25"/>
     </row>
-    <row r="18" spans="1:6">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A18" s="19"/>
       <c r="B18" s="18">
         <v>75</v>
       </c>
       <c r="F18" s="25"/>
     </row>
-    <row r="19" spans="1:6">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A19" s="20"/>
       <c r="B19" s="21">
         <v>80</v>
@@ -5732,4 +5790,1866 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{429AE0B6-F526-4890-BA9C-B271CEA32A02}">
+  <dimension ref="A1:H167"/>
+  <sheetFormatPr defaultRowHeight="16" x14ac:dyDescent="0.4"/>
+  <cols>
+    <col min="1" max="1" width="13.453125" style="34" customWidth="1"/>
+    <col min="2" max="2" width="14.6328125" style="34" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.6328125" style="34" bestFit="1" customWidth="1"/>
+    <col min="4" max="16384" width="8.7265625" style="34"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" ht="30" x14ac:dyDescent="0.4">
+      <c r="A1" s="33" t="s">
+        <v>17</v>
+      </c>
+      <c r="B1" s="33" t="s">
+        <v>18</v>
+      </c>
+      <c r="C1" s="33" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="105" x14ac:dyDescent="0.4">
+      <c r="A2" s="35">
+        <v>280</v>
+      </c>
+      <c r="B2" s="36">
+        <v>3.6030000000000002E-19</v>
+      </c>
+      <c r="C2" s="36">
+        <v>1.2689999999999999E-4</v>
+      </c>
+      <c r="E2" s="33" t="s">
+        <v>20</v>
+      </c>
+      <c r="F2" s="33" t="s">
+        <v>21</v>
+      </c>
+      <c r="G2" s="33" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A3" s="35">
+        <v>285</v>
+      </c>
+      <c r="B3" s="36">
+        <v>9.2059999999999993E-13</v>
+      </c>
+      <c r="C3" s="35">
+        <v>660</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A4" s="35">
+        <v>290</v>
+      </c>
+      <c r="B4" s="36">
+        <v>6.4760000000000005E-8</v>
+      </c>
+      <c r="C4" s="36">
+        <v>47240000</v>
+      </c>
+      <c r="H4" s="34" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A5" s="35">
+        <v>295</v>
+      </c>
+      <c r="B5" s="36">
+        <v>3.625E-5</v>
+      </c>
+      <c r="C5" s="36">
+        <v>26940000000</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A6" s="35">
+        <v>300</v>
+      </c>
+      <c r="B6" s="36">
+        <v>1.3940000000000001E-3</v>
+      </c>
+      <c r="C6" s="36">
+        <v>1079000000000</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A7" s="35">
+        <v>305</v>
+      </c>
+      <c r="B7" s="36">
+        <v>1.5970000000000002E-2</v>
+      </c>
+      <c r="C7" s="36">
+        <v>13330000000000</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A8" s="35">
+        <v>310</v>
+      </c>
+      <c r="B8" s="36">
+        <v>6.0539999999999997E-2</v>
+      </c>
+      <c r="C8" s="36">
+        <v>60540000000000</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A9" s="35">
+        <v>315</v>
+      </c>
+      <c r="B9" s="35">
+        <v>0.13009999999999999</v>
+      </c>
+      <c r="C9" s="36">
+        <v>163700000000000</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A10" s="35">
+        <v>320</v>
+      </c>
+      <c r="B10" s="35">
+        <v>0.21179999999999999</v>
+      </c>
+      <c r="C10" s="36">
+        <v>334100000000000</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A11" s="35">
+        <v>325</v>
+      </c>
+      <c r="B11" s="35">
+        <v>0.31019999999999998</v>
+      </c>
+      <c r="C11" s="36">
+        <v>587700000000000</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A12" s="35">
+        <v>330</v>
+      </c>
+      <c r="B12" s="35">
+        <v>0.41710000000000003</v>
+      </c>
+      <c r="C12" s="36">
+        <v>933900000000000</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A13" s="35">
+        <v>335</v>
+      </c>
+      <c r="B13" s="35">
+        <v>0.4194</v>
+      </c>
+      <c r="C13" s="36">
+        <v>1287000000000000</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A14" s="35">
+        <v>340</v>
+      </c>
+      <c r="B14" s="35">
+        <v>0.47</v>
+      </c>
+      <c r="C14" s="36">
+        <v>1689000000000000</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A15" s="35">
+        <v>345</v>
+      </c>
+      <c r="B15" s="35">
+        <v>0.4708</v>
+      </c>
+      <c r="C15" s="36">
+        <v>2098000000000000</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A16" s="35">
+        <v>350</v>
+      </c>
+      <c r="B16" s="35">
+        <v>0.50660000000000005</v>
+      </c>
+      <c r="C16" s="36">
+        <v>2544000000000000</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A17" s="35">
+        <v>355</v>
+      </c>
+      <c r="B17" s="35">
+        <v>0.55020000000000002</v>
+      </c>
+      <c r="C17" s="36">
+        <v>3035000000000000</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A18" s="35">
+        <v>360</v>
+      </c>
+      <c r="B18" s="35">
+        <v>0.5101</v>
+      </c>
+      <c r="C18" s="36">
+        <v>3497000000000000</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A19" s="35">
+        <v>365</v>
+      </c>
+      <c r="B19" s="35">
+        <v>0.65269999999999995</v>
+      </c>
+      <c r="C19" s="36">
+        <v>4096000000000000</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A20" s="35">
+        <v>370</v>
+      </c>
+      <c r="B20" s="35">
+        <v>0.69510000000000005</v>
+      </c>
+      <c r="C20" s="36">
+        <v>4743000000000000</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A21" s="35">
+        <v>375</v>
+      </c>
+      <c r="B21" s="35">
+        <v>0.62790000000000001</v>
+      </c>
+      <c r="C21" s="36">
+        <v>5335000000000000</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A22" s="35">
+        <v>380</v>
+      </c>
+      <c r="B22" s="35">
+        <v>0.72230000000000005</v>
+      </c>
+      <c r="C22" s="36">
+        <v>6026000000000000</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A23" s="35">
+        <v>385</v>
+      </c>
+      <c r="B23" s="35">
+        <v>0.58130000000000004</v>
+      </c>
+      <c r="C23" s="36">
+        <v>6589000000000000</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A24" s="35">
+        <v>390</v>
+      </c>
+      <c r="B24" s="35">
+        <v>0.74550000000000005</v>
+      </c>
+      <c r="C24" s="36">
+        <v>7320000000000000</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A25" s="35">
+        <v>395</v>
+      </c>
+      <c r="B25" s="35">
+        <v>0.60699999999999998</v>
+      </c>
+      <c r="C25" s="36">
+        <v>7923000000000000</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A26" s="35">
+        <v>400</v>
+      </c>
+      <c r="B26" s="35">
+        <v>1.071</v>
+      </c>
+      <c r="C26" s="36">
+        <v>9001000000000000</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A27" s="35">
+        <v>405</v>
+      </c>
+      <c r="B27" s="35">
+        <v>1.1439999999999999</v>
+      </c>
+      <c r="C27" s="36">
+        <v>1.017E+16</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A28" s="35">
+        <v>410</v>
+      </c>
+      <c r="B28" s="35">
+        <v>1.1659999999999999</v>
+      </c>
+      <c r="C28" s="36">
+        <v>1.137E+16</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A29" s="35">
+        <v>415</v>
+      </c>
+      <c r="B29" s="35">
+        <v>1.216</v>
+      </c>
+      <c r="C29" s="36">
+        <v>1.264E+16</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A30" s="35">
+        <v>420</v>
+      </c>
+      <c r="B30" s="35">
+        <v>1.2070000000000001</v>
+      </c>
+      <c r="C30" s="36">
+        <v>1.391E+16</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A31" s="35">
+        <v>425</v>
+      </c>
+      <c r="B31" s="35">
+        <v>1.2110000000000001</v>
+      </c>
+      <c r="C31" s="36">
+        <v>1.521E+16</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A32" s="35">
+        <v>430</v>
+      </c>
+      <c r="B32" s="35">
+        <v>1.048</v>
+      </c>
+      <c r="C32" s="36">
+        <v>1.634E+16</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A33" s="35">
+        <v>435</v>
+      </c>
+      <c r="B33" s="35">
+        <v>1.268</v>
+      </c>
+      <c r="C33" s="36">
+        <v>1.773E+16</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A34" s="35">
+        <v>440</v>
+      </c>
+      <c r="B34" s="35">
+        <v>1.3029999999999999</v>
+      </c>
+      <c r="C34" s="36">
+        <v>1.917E+16</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A35" s="35">
+        <v>445</v>
+      </c>
+      <c r="B35" s="35">
+        <v>1.42</v>
+      </c>
+      <c r="C35" s="36">
+        <v>2.076E+16</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A36" s="35">
+        <v>450</v>
+      </c>
+      <c r="B36" s="35">
+        <v>1.5389999999999999</v>
+      </c>
+      <c r="C36" s="36">
+        <v>2.25E+16</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A37" s="35">
+        <v>455</v>
+      </c>
+      <c r="B37" s="35">
+        <v>1.528</v>
+      </c>
+      <c r="C37" s="36">
+        <v>2.425E+16</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A38" s="35">
+        <v>460</v>
+      </c>
+      <c r="B38" s="35">
+        <v>1.5549999999999999</v>
+      </c>
+      <c r="C38" s="36">
+        <v>2.605E+16</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A39" s="35">
+        <v>465</v>
+      </c>
+      <c r="B39" s="35">
+        <v>1.548</v>
+      </c>
+      <c r="C39" s="36">
+        <v>2.786E+16</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A40" s="35">
+        <v>470</v>
+      </c>
+      <c r="B40" s="35">
+        <v>1.5489999999999999</v>
+      </c>
+      <c r="C40" s="36">
+        <v>2.969E+16</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A41" s="35">
+        <v>475</v>
+      </c>
+      <c r="B41" s="35">
+        <v>1.573</v>
+      </c>
+      <c r="C41" s="36">
+        <v>3.157E+16</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A42" s="35">
+        <v>480</v>
+      </c>
+      <c r="B42" s="35">
+        <v>1.6080000000000001</v>
+      </c>
+      <c r="C42" s="36">
+        <v>3.351E+16</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A43" s="35">
+        <v>485</v>
+      </c>
+      <c r="B43" s="35">
+        <v>1.488</v>
+      </c>
+      <c r="C43" s="36">
+        <v>3.533E+16</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A44" s="35">
+        <v>490</v>
+      </c>
+      <c r="B44" s="35">
+        <v>1.53</v>
+      </c>
+      <c r="C44" s="36">
+        <v>3.721E+16</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A45" s="35">
+        <v>495</v>
+      </c>
+      <c r="B45" s="35">
+        <v>1.5820000000000001</v>
+      </c>
+      <c r="C45" s="36">
+        <v>3.918E+16</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A46" s="35">
+        <v>500</v>
+      </c>
+      <c r="B46" s="35">
+        <v>1.5269999999999999</v>
+      </c>
+      <c r="C46" s="36">
+        <v>4.11E+16</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A47" s="35">
+        <v>505</v>
+      </c>
+      <c r="B47" s="35">
+        <v>1.5449999999999999</v>
+      </c>
+      <c r="C47" s="36">
+        <v>4.307E+16</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A48" s="35">
+        <v>510</v>
+      </c>
+      <c r="B48" s="35">
+        <v>1.5609999999999999</v>
+      </c>
+      <c r="C48" s="36">
+        <v>4.507E+16</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A49" s="35">
+        <v>515</v>
+      </c>
+      <c r="B49" s="35">
+        <v>1.4730000000000001</v>
+      </c>
+      <c r="C49" s="36">
+        <v>4.698E+16</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A50" s="35">
+        <v>520</v>
+      </c>
+      <c r="B50" s="35">
+        <v>1.4810000000000001</v>
+      </c>
+      <c r="C50" s="36">
+        <v>4.891E+16</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A51" s="35">
+        <v>525</v>
+      </c>
+      <c r="B51" s="35">
+        <v>1.5069999999999999</v>
+      </c>
+      <c r="C51" s="36">
+        <v>5.09E+16</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A52" s="35">
+        <v>530</v>
+      </c>
+      <c r="B52" s="35">
+        <v>1.569</v>
+      </c>
+      <c r="C52" s="36">
+        <v>5.3E+16</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A53" s="35">
+        <v>535</v>
+      </c>
+      <c r="B53" s="35">
+        <v>1.5289999999999999</v>
+      </c>
+      <c r="C53" s="36">
+        <v>5.505E+16</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A54" s="35">
+        <v>540</v>
+      </c>
+      <c r="B54" s="35">
+        <v>1.5069999999999999</v>
+      </c>
+      <c r="C54" s="36">
+        <v>5.71E+16</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A55" s="35">
+        <v>545</v>
+      </c>
+      <c r="B55" s="35">
+        <v>1.538</v>
+      </c>
+      <c r="C55" s="36">
+        <v>5.921E+16</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A56" s="35">
+        <v>550</v>
+      </c>
+      <c r="B56" s="35">
+        <v>1.538</v>
+      </c>
+      <c r="C56" s="36">
+        <v>6.134E+16</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A57" s="35">
+        <v>555</v>
+      </c>
+      <c r="B57" s="35">
+        <v>1.532</v>
+      </c>
+      <c r="C57" s="36">
+        <v>6.348E+16</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A58" s="35">
+        <v>560</v>
+      </c>
+      <c r="B58" s="35">
+        <v>1.4970000000000001</v>
+      </c>
+      <c r="C58" s="36">
+        <v>6.558E+16</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A59" s="35">
+        <v>565</v>
+      </c>
+      <c r="B59" s="35">
+        <v>1.504</v>
+      </c>
+      <c r="C59" s="36">
+        <v>6.772E+16</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A60" s="35">
+        <v>570</v>
+      </c>
+      <c r="B60" s="35">
+        <v>1.4830000000000001</v>
+      </c>
+      <c r="C60" s="36">
+        <v>6.985E+16</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A61" s="35">
+        <v>575</v>
+      </c>
+      <c r="B61" s="35">
+        <v>1.4910000000000001</v>
+      </c>
+      <c r="C61" s="36">
+        <v>7.2E+16</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A62" s="35">
+        <v>580</v>
+      </c>
+      <c r="B62" s="35">
+        <v>1.492</v>
+      </c>
+      <c r="C62" s="36">
+        <v>7.418E+16</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A63" s="35">
+        <v>585</v>
+      </c>
+      <c r="B63" s="35">
+        <v>1.5229999999999999</v>
+      </c>
+      <c r="C63" s="36">
+        <v>7.642E+16</v>
+      </c>
+    </row>
+    <row r="64" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A64" s="35">
+        <v>590</v>
+      </c>
+      <c r="B64" s="35">
+        <v>1.409</v>
+      </c>
+      <c r="C64" s="36">
+        <v>7.851E+16</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A65" s="35">
+        <v>595</v>
+      </c>
+      <c r="B65" s="35">
+        <v>1.4510000000000001</v>
+      </c>
+      <c r="C65" s="36">
+        <v>8.068E+16</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A66" s="35">
+        <v>600</v>
+      </c>
+      <c r="B66" s="35">
+        <v>1.4550000000000001</v>
+      </c>
+      <c r="C66" s="36">
+        <v>8.288E+16</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A67" s="35">
+        <v>605</v>
+      </c>
+      <c r="B67" s="35">
+        <v>1.4810000000000001</v>
+      </c>
+      <c r="C67" s="36">
+        <v>8.513E+16</v>
+      </c>
+    </row>
+    <row r="68" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A68" s="35">
+        <v>610</v>
+      </c>
+      <c r="B68" s="35">
+        <v>1.47</v>
+      </c>
+      <c r="C68" s="36">
+        <v>8.739E+16</v>
+      </c>
+    </row>
+    <row r="69" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A69" s="35">
+        <v>615</v>
+      </c>
+      <c r="B69" s="35">
+        <v>1.4379999999999999</v>
+      </c>
+      <c r="C69" s="36">
+        <v>8.961E+16</v>
+      </c>
+    </row>
+    <row r="70" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A70" s="35">
+        <v>620</v>
+      </c>
+      <c r="B70" s="35">
+        <v>1.4590000000000001</v>
+      </c>
+      <c r="C70" s="36">
+        <v>9.189E+16</v>
+      </c>
+    </row>
+    <row r="71" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A71" s="35">
+        <v>625</v>
+      </c>
+      <c r="B71" s="35">
+        <v>1.41</v>
+      </c>
+      <c r="C71" s="36">
+        <v>9.41E+16</v>
+      </c>
+    </row>
+    <row r="72" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A72" s="35">
+        <v>630</v>
+      </c>
+      <c r="B72" s="35">
+        <v>1.39</v>
+      </c>
+      <c r="C72" s="36">
+        <v>9.631E+16</v>
+      </c>
+    </row>
+    <row r="73" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A73" s="35">
+        <v>635</v>
+      </c>
+      <c r="B73" s="35">
+        <v>1.4339999999999999</v>
+      </c>
+      <c r="C73" s="36">
+        <v>9.86E+16</v>
+      </c>
+    </row>
+    <row r="74" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A74" s="35">
+        <v>640</v>
+      </c>
+      <c r="B74" s="35">
+        <v>1.444</v>
+      </c>
+      <c r="C74" s="36">
+        <v>1.009E+17</v>
+      </c>
+    </row>
+    <row r="75" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A75" s="35">
+        <v>645</v>
+      </c>
+      <c r="B75" s="35">
+        <v>1.429</v>
+      </c>
+      <c r="C75" s="36">
+        <v>1.032E+17</v>
+      </c>
+    </row>
+    <row r="76" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A76" s="35">
+        <v>650</v>
+      </c>
+      <c r="B76" s="35">
+        <v>1.3859999999999999</v>
+      </c>
+      <c r="C76" s="36">
+        <v>1.055E+17</v>
+      </c>
+    </row>
+    <row r="77" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A77" s="35">
+        <v>655</v>
+      </c>
+      <c r="B77" s="35">
+        <v>1.3240000000000001</v>
+      </c>
+      <c r="C77" s="36">
+        <v>1.077E+17</v>
+      </c>
+    </row>
+    <row r="78" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A78" s="35">
+        <v>660</v>
+      </c>
+      <c r="B78" s="35">
+        <v>1.385</v>
+      </c>
+      <c r="C78" s="36">
+        <v>1.1E+17</v>
+      </c>
+    </row>
+    <row r="79" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A79" s="35">
+        <v>665</v>
+      </c>
+      <c r="B79" s="35">
+        <v>1.4039999999999999</v>
+      </c>
+      <c r="C79" s="36">
+        <v>1.123E+17</v>
+      </c>
+    </row>
+    <row r="80" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A80" s="35">
+        <v>670</v>
+      </c>
+      <c r="B80" s="35">
+        <v>1.415</v>
+      </c>
+      <c r="C80" s="36">
+        <v>1.147E+17</v>
+      </c>
+    </row>
+    <row r="81" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A81" s="35">
+        <v>675</v>
+      </c>
+      <c r="B81" s="35">
+        <v>1.4019999999999999</v>
+      </c>
+      <c r="C81" s="36">
+        <v>1.171E+17</v>
+      </c>
+    </row>
+    <row r="82" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A82" s="35">
+        <v>680</v>
+      </c>
+      <c r="B82" s="35">
+        <v>1.3919999999999999</v>
+      </c>
+      <c r="C82" s="36">
+        <v>1.195E+17</v>
+      </c>
+    </row>
+    <row r="83" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A83" s="35">
+        <v>685</v>
+      </c>
+      <c r="B83" s="35">
+        <v>1.2889999999999999</v>
+      </c>
+      <c r="C83" s="36">
+        <v>1.217E+17</v>
+      </c>
+    </row>
+    <row r="84" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A84" s="35">
+        <v>690</v>
+      </c>
+      <c r="B84" s="35">
+        <v>1.18</v>
+      </c>
+      <c r="C84" s="36">
+        <v>1.238E+17</v>
+      </c>
+    </row>
+    <row r="85" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A85" s="35">
+        <v>695</v>
+      </c>
+      <c r="B85" s="35">
+        <v>1.274</v>
+      </c>
+      <c r="C85" s="36">
+        <v>1.26E+17</v>
+      </c>
+    </row>
+    <row r="86" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A86" s="35">
+        <v>700</v>
+      </c>
+      <c r="B86" s="35">
+        <v>1.2829999999999999</v>
+      </c>
+      <c r="C86" s="36">
+        <v>1.282E+17</v>
+      </c>
+    </row>
+    <row r="87" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A87" s="35">
+        <v>705</v>
+      </c>
+      <c r="B87" s="35">
+        <v>1.302</v>
+      </c>
+      <c r="C87" s="36">
+        <v>1.305E+17</v>
+      </c>
+    </row>
+    <row r="88" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A88" s="35">
+        <v>710</v>
+      </c>
+      <c r="B88" s="35">
+        <v>1.306</v>
+      </c>
+      <c r="C88" s="36">
+        <v>1.329E+17</v>
+      </c>
+    </row>
+    <row r="89" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A89" s="35">
+        <v>715</v>
+      </c>
+      <c r="B89" s="35">
+        <v>1.2430000000000001</v>
+      </c>
+      <c r="C89" s="36">
+        <v>1.351E+17</v>
+      </c>
+    </row>
+    <row r="90" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A90" s="35">
+        <v>720</v>
+      </c>
+      <c r="B90" s="35">
+        <v>1.05</v>
+      </c>
+      <c r="C90" s="36">
+        <v>1.37E+17</v>
+      </c>
+    </row>
+    <row r="91" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A91" s="35">
+        <v>725</v>
+      </c>
+      <c r="B91" s="35">
+        <v>1.08</v>
+      </c>
+      <c r="C91" s="36">
+        <v>1.39E+17</v>
+      </c>
+    </row>
+    <row r="92" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A92" s="35">
+        <v>730</v>
+      </c>
+      <c r="B92" s="35">
+        <v>1.0880000000000001</v>
+      </c>
+      <c r="C92" s="36">
+        <v>1.41E+17</v>
+      </c>
+    </row>
+    <row r="93" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A93" s="35">
+        <v>735</v>
+      </c>
+      <c r="B93" s="35">
+        <v>1.206</v>
+      </c>
+      <c r="C93" s="36">
+        <v>1.432E+17</v>
+      </c>
+    </row>
+    <row r="94" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A94" s="35">
+        <v>740</v>
+      </c>
+      <c r="B94" s="35">
+        <v>1.21</v>
+      </c>
+      <c r="C94" s="36">
+        <v>1.455E+17</v>
+      </c>
+    </row>
+    <row r="95" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A95" s="35">
+        <v>745</v>
+      </c>
+      <c r="B95" s="35">
+        <v>1.2430000000000001</v>
+      </c>
+      <c r="C95" s="36">
+        <v>1.478E+17</v>
+      </c>
+    </row>
+    <row r="96" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A96" s="35">
+        <v>750</v>
+      </c>
+      <c r="B96" s="35">
+        <v>1.232</v>
+      </c>
+      <c r="C96" s="36">
+        <v>1.501E+17</v>
+      </c>
+    </row>
+    <row r="97" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A97" s="35">
+        <v>755</v>
+      </c>
+      <c r="B97" s="35">
+        <v>1.2270000000000001</v>
+      </c>
+      <c r="C97" s="36">
+        <v>1.524E+17</v>
+      </c>
+    </row>
+    <row r="98" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A98" s="35">
+        <v>760</v>
+      </c>
+      <c r="B98" s="35">
+        <v>0.69710000000000005</v>
+      </c>
+      <c r="C98" s="36">
+        <v>1.538E+17</v>
+      </c>
+    </row>
+    <row r="99" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A99" s="35">
+        <v>765</v>
+      </c>
+      <c r="B99" s="35">
+        <v>0.68759999999999999</v>
+      </c>
+      <c r="C99" s="36">
+        <v>1.551E+17</v>
+      </c>
+    </row>
+    <row r="100" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A100" s="35">
+        <v>770</v>
+      </c>
+      <c r="B100" s="35">
+        <v>1.143</v>
+      </c>
+      <c r="C100" s="36">
+        <v>1.573E+17</v>
+      </c>
+    </row>
+    <row r="101" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A101" s="35">
+        <v>775</v>
+      </c>
+      <c r="B101" s="35">
+        <v>1.1719999999999999</v>
+      </c>
+      <c r="C101" s="36">
+        <v>1.596E+17</v>
+      </c>
+    </row>
+    <row r="102" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A102" s="35">
+        <v>780</v>
+      </c>
+      <c r="B102" s="35">
+        <v>1.1639999999999999</v>
+      </c>
+      <c r="C102" s="36">
+        <v>1.619E+17</v>
+      </c>
+    </row>
+    <row r="103" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A103" s="35">
+        <v>785</v>
+      </c>
+      <c r="B103" s="35">
+        <v>1.1539999999999999</v>
+      </c>
+      <c r="C103" s="36">
+        <v>1.642E+17</v>
+      </c>
+    </row>
+    <row r="104" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A104" s="35">
+        <v>790</v>
+      </c>
+      <c r="B104" s="35">
+        <v>1.1060000000000001</v>
+      </c>
+      <c r="C104" s="36">
+        <v>1.664E+17</v>
+      </c>
+    </row>
+    <row r="105" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A105" s="35">
+        <v>795</v>
+      </c>
+      <c r="B105" s="35">
+        <v>1.085</v>
+      </c>
+      <c r="C105" s="36">
+        <v>1.685E+17</v>
+      </c>
+    </row>
+    <row r="106" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A106" s="35">
+        <v>800</v>
+      </c>
+      <c r="B106" s="35">
+        <v>1.085</v>
+      </c>
+      <c r="C106" s="36">
+        <v>1.707E+17</v>
+      </c>
+    </row>
+    <row r="107" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A107" s="35">
+        <v>805</v>
+      </c>
+      <c r="B107" s="35">
+        <v>1.073</v>
+      </c>
+      <c r="C107" s="36">
+        <v>1.729E+17</v>
+      </c>
+    </row>
+    <row r="108" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A108" s="35">
+        <v>810</v>
+      </c>
+      <c r="B108" s="35">
+        <v>1.05</v>
+      </c>
+      <c r="C108" s="36">
+        <v>1.75E+17</v>
+      </c>
+    </row>
+    <row r="109" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A109" s="35">
+        <v>815</v>
+      </c>
+      <c r="B109" s="35">
+        <v>0.89610000000000001</v>
+      </c>
+      <c r="C109" s="36">
+        <v>1.769E+17</v>
+      </c>
+    </row>
+    <row r="110" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A110" s="35">
+        <v>820</v>
+      </c>
+      <c r="B110" s="35">
+        <v>0.89900000000000002</v>
+      </c>
+      <c r="C110" s="36">
+        <v>1.787E+17</v>
+      </c>
+    </row>
+    <row r="111" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A111" s="35">
+        <v>825</v>
+      </c>
+      <c r="B111" s="35">
+        <v>0.9002</v>
+      </c>
+      <c r="C111" s="36">
+        <v>1.806E+17</v>
+      </c>
+    </row>
+    <row r="112" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A112" s="35">
+        <v>830</v>
+      </c>
+      <c r="B112" s="35">
+        <v>0.90490000000000004</v>
+      </c>
+      <c r="C112" s="36">
+        <v>1.825E+17</v>
+      </c>
+    </row>
+    <row r="113" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A113" s="35">
+        <v>835</v>
+      </c>
+      <c r="B113" s="35">
+        <v>0.97109999999999996</v>
+      </c>
+      <c r="C113" s="36">
+        <v>1.845E+17</v>
+      </c>
+    </row>
+    <row r="114" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A114" s="35">
+        <v>840</v>
+      </c>
+      <c r="B114" s="35">
+        <v>1.002</v>
+      </c>
+      <c r="C114" s="36">
+        <v>1.866E+17</v>
+      </c>
+    </row>
+    <row r="115" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A115" s="35">
+        <v>845</v>
+      </c>
+      <c r="B115" s="35">
+        <v>1</v>
+      </c>
+      <c r="C115" s="36">
+        <v>1.888E+17</v>
+      </c>
+    </row>
+    <row r="116" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A116" s="35">
+        <v>850</v>
+      </c>
+      <c r="B116" s="35">
+        <v>0.96030000000000004</v>
+      </c>
+      <c r="C116" s="36">
+        <v>1.908E+17</v>
+      </c>
+    </row>
+    <row r="117" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A117" s="35">
+        <v>855</v>
+      </c>
+      <c r="B117" s="35">
+        <v>0.93610000000000004</v>
+      </c>
+      <c r="C117" s="36">
+        <v>1.928E+17</v>
+      </c>
+    </row>
+    <row r="118" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A118" s="35">
+        <v>860</v>
+      </c>
+      <c r="B118" s="35">
+        <v>0.98799999999999999</v>
+      </c>
+      <c r="C118" s="36">
+        <v>1.95E+17</v>
+      </c>
+    </row>
+    <row r="119" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A119" s="35">
+        <v>865</v>
+      </c>
+      <c r="B119" s="35">
+        <v>0.93969999999999998</v>
+      </c>
+      <c r="C119" s="36">
+        <v>1.97E+17</v>
+      </c>
+    </row>
+    <row r="120" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A120" s="35">
+        <v>870</v>
+      </c>
+      <c r="B120" s="35">
+        <v>0.95530000000000004</v>
+      </c>
+      <c r="C120" s="36">
+        <v>1.991E+17</v>
+      </c>
+    </row>
+    <row r="121" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A121" s="35">
+        <v>875</v>
+      </c>
+      <c r="B121" s="35">
+        <v>0.94399999999999995</v>
+      </c>
+      <c r="C121" s="36">
+        <v>2.012E+17</v>
+      </c>
+    </row>
+    <row r="122" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A122" s="35">
+        <v>880</v>
+      </c>
+      <c r="B122" s="35">
+        <v>0.93140000000000001</v>
+      </c>
+      <c r="C122" s="36">
+        <v>2.032E+17</v>
+      </c>
+    </row>
+    <row r="123" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A123" s="35">
+        <v>885</v>
+      </c>
+      <c r="B123" s="35">
+        <v>0.92279999999999995</v>
+      </c>
+      <c r="C123" s="36">
+        <v>2.053E+17</v>
+      </c>
+    </row>
+    <row r="124" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A124" s="35">
+        <v>890</v>
+      </c>
+      <c r="B124" s="35">
+        <v>0.91920000000000002</v>
+      </c>
+      <c r="C124" s="36">
+        <v>2.073E+17</v>
+      </c>
+    </row>
+    <row r="125" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A125" s="35">
+        <v>895</v>
+      </c>
+      <c r="B125" s="35">
+        <v>0.79320000000000002</v>
+      </c>
+      <c r="C125" s="36">
+        <v>2.091E+17</v>
+      </c>
+    </row>
+    <row r="126" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A126" s="35">
+        <v>900</v>
+      </c>
+      <c r="B126" s="35">
+        <v>0.65259999999999996</v>
+      </c>
+      <c r="C126" s="36">
+        <v>2.106E+17</v>
+      </c>
+    </row>
+    <row r="127" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A127" s="35">
+        <v>905</v>
+      </c>
+      <c r="B127" s="35">
+        <v>0.75060000000000004</v>
+      </c>
+      <c r="C127" s="36">
+        <v>2.123E+17</v>
+      </c>
+    </row>
+    <row r="128" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A128" s="35">
+        <v>910</v>
+      </c>
+      <c r="B128" s="35">
+        <v>0.66379999999999995</v>
+      </c>
+      <c r="C128" s="36">
+        <v>2.138E+17</v>
+      </c>
+    </row>
+    <row r="129" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A129" s="35">
+        <v>915</v>
+      </c>
+      <c r="B129" s="35">
+        <v>0.64429999999999998</v>
+      </c>
+      <c r="C129" s="36">
+        <v>2.153E+17</v>
+      </c>
+    </row>
+    <row r="130" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A130" s="35">
+        <v>920</v>
+      </c>
+      <c r="B130" s="35">
+        <v>0.71379999999999999</v>
+      </c>
+      <c r="C130" s="36">
+        <v>2.17E+17</v>
+      </c>
+    </row>
+    <row r="131" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A131" s="35">
+        <v>925</v>
+      </c>
+      <c r="B131" s="35">
+        <v>0.72540000000000004</v>
+      </c>
+      <c r="C131" s="36">
+        <v>2.187E+17</v>
+      </c>
+    </row>
+    <row r="132" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A132" s="35">
+        <v>930</v>
+      </c>
+      <c r="B132" s="35">
+        <v>0.45900000000000002</v>
+      </c>
+      <c r="C132" s="36">
+        <v>2.197E+17</v>
+      </c>
+    </row>
+    <row r="133" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A133" s="35">
+        <v>935</v>
+      </c>
+      <c r="B133" s="35">
+        <v>0.19520000000000001</v>
+      </c>
+      <c r="C133" s="36">
+        <v>2.202E+17</v>
+      </c>
+    </row>
+    <row r="134" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A134" s="35">
+        <v>940</v>
+      </c>
+      <c r="B134" s="35">
+        <v>0.36449999999999999</v>
+      </c>
+      <c r="C134" s="36">
+        <v>2.211E+17</v>
+      </c>
+    </row>
+    <row r="135" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A135" s="35">
+        <v>945</v>
+      </c>
+      <c r="B135" s="35">
+        <v>0.29949999999999999</v>
+      </c>
+      <c r="C135" s="36">
+        <v>2.218E+17</v>
+      </c>
+    </row>
+    <row r="136" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A136" s="35">
+        <v>950</v>
+      </c>
+      <c r="B136" s="35">
+        <v>0.33689999999999998</v>
+      </c>
+      <c r="C136" s="36">
+        <v>2.226E+17</v>
+      </c>
+    </row>
+    <row r="137" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A137" s="35">
+        <v>955</v>
+      </c>
+      <c r="B137" s="35">
+        <v>0.34350000000000003</v>
+      </c>
+      <c r="C137" s="36">
+        <v>2.234E+17</v>
+      </c>
+    </row>
+    <row r="138" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A138" s="35">
+        <v>960</v>
+      </c>
+      <c r="B138" s="35">
+        <v>0.4274</v>
+      </c>
+      <c r="C138" s="36">
+        <v>2.244E+17</v>
+      </c>
+    </row>
+    <row r="139" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A139" s="35">
+        <v>965</v>
+      </c>
+      <c r="B139" s="35">
+        <v>0.49519999999999997</v>
+      </c>
+      <c r="C139" s="36">
+        <v>2.256E+17</v>
+      </c>
+    </row>
+    <row r="140" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A140" s="35">
+        <v>970</v>
+      </c>
+      <c r="B140" s="35">
+        <v>0.6673</v>
+      </c>
+      <c r="C140" s="36">
+        <v>2.273E+17</v>
+      </c>
+    </row>
+    <row r="141" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A141" s="35">
+        <v>975</v>
+      </c>
+      <c r="B141" s="35">
+        <v>0.59619999999999995</v>
+      </c>
+      <c r="C141" s="36">
+        <v>2.287E+17</v>
+      </c>
+    </row>
+    <row r="142" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A142" s="35">
+        <v>980</v>
+      </c>
+      <c r="B142" s="35">
+        <v>0.65059999999999996</v>
+      </c>
+      <c r="C142" s="36">
+        <v>2.303E+17</v>
+      </c>
+    </row>
+    <row r="143" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A143" s="35">
+        <v>985</v>
+      </c>
+      <c r="B143" s="35">
+        <v>0.71530000000000005</v>
+      </c>
+      <c r="C143" s="36">
+        <v>2.321E+17</v>
+      </c>
+    </row>
+    <row r="144" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A144" s="35">
+        <v>990</v>
+      </c>
+      <c r="B144" s="35">
+        <v>0.74180000000000001</v>
+      </c>
+      <c r="C144" s="36">
+        <v>2.339E+17</v>
+      </c>
+    </row>
+    <row r="145" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A145" s="35">
+        <v>995</v>
+      </c>
+      <c r="B145" s="35">
+        <v>0.74470000000000003</v>
+      </c>
+      <c r="C145" s="36">
+        <v>2.358E+17</v>
+      </c>
+    </row>
+    <row r="146" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A146" s="35">
+        <v>1000</v>
+      </c>
+      <c r="B146" s="35">
+        <v>0.73499999999999999</v>
+      </c>
+      <c r="C146" s="36">
+        <v>2.377E+17</v>
+      </c>
+    </row>
+    <row r="147" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A147" s="35">
+        <v>1005</v>
+      </c>
+      <c r="B147" s="35">
+        <v>0.7137</v>
+      </c>
+      <c r="C147" s="36">
+        <v>2.395E+17</v>
+      </c>
+    </row>
+    <row r="148" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A148" s="35">
+        <v>1010</v>
+      </c>
+      <c r="B148" s="35">
+        <v>0.71960000000000002</v>
+      </c>
+      <c r="C148" s="36">
+        <v>2.413E+17</v>
+      </c>
+    </row>
+    <row r="149" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A149" s="35">
+        <v>1015</v>
+      </c>
+      <c r="B149" s="35">
+        <v>0.71050000000000002</v>
+      </c>
+      <c r="C149" s="36">
+        <v>2.431E+17</v>
+      </c>
+    </row>
+    <row r="150" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A150" s="35">
+        <v>1020</v>
+      </c>
+      <c r="B150" s="35">
+        <v>0.69669999999999999</v>
+      </c>
+      <c r="C150" s="36">
+        <v>2.449E+17</v>
+      </c>
+    </row>
+    <row r="151" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A151" s="35">
+        <v>1025</v>
+      </c>
+      <c r="B151" s="35">
+        <v>0.6925</v>
+      </c>
+      <c r="C151" s="36">
+        <v>2.467E+17</v>
+      </c>
+    </row>
+    <row r="152" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A152" s="35">
+        <v>1030</v>
+      </c>
+      <c r="B152" s="35">
+        <v>0.68689999999999996</v>
+      </c>
+      <c r="C152" s="36">
+        <v>2.485E+17</v>
+      </c>
+    </row>
+    <row r="153" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A153" s="35">
+        <v>1035</v>
+      </c>
+      <c r="B153" s="35">
+        <v>0.67720000000000002</v>
+      </c>
+      <c r="C153" s="36">
+        <v>2.502E+17</v>
+      </c>
+    </row>
+    <row r="154" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A154" s="35">
+        <v>1040</v>
+      </c>
+      <c r="B154" s="35">
+        <v>0.67069999999999996</v>
+      </c>
+      <c r="C154" s="36">
+        <v>2.52E+17</v>
+      </c>
+    </row>
+    <row r="155" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A155" s="35">
+        <v>1045</v>
+      </c>
+      <c r="B155" s="35">
+        <v>0.65869999999999995</v>
+      </c>
+      <c r="C155" s="36">
+        <v>2.537E+17</v>
+      </c>
+    </row>
+    <row r="156" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A156" s="35">
+        <v>1050</v>
+      </c>
+      <c r="B156" s="35">
+        <v>0.65439999999999998</v>
+      </c>
+      <c r="C156" s="36">
+        <v>2.554E+17</v>
+      </c>
+    </row>
+    <row r="157" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A157" s="35">
+        <v>1055</v>
+      </c>
+      <c r="B157" s="35">
+        <v>0.64529999999999998</v>
+      </c>
+      <c r="C157" s="36">
+        <v>2.571E+17</v>
+      </c>
+    </row>
+    <row r="158" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A158" s="35">
+        <v>1060</v>
+      </c>
+      <c r="B158" s="35">
+        <v>0.62729999999999997</v>
+      </c>
+      <c r="C158" s="36">
+        <v>2.588E+17</v>
+      </c>
+    </row>
+    <row r="159" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A159" s="35">
+        <v>1065</v>
+      </c>
+      <c r="B159" s="35">
+        <v>0.62260000000000004</v>
+      </c>
+      <c r="C159" s="36">
+        <v>2.605E+17</v>
+      </c>
+    </row>
+    <row r="160" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A160" s="35">
+        <v>1070</v>
+      </c>
+      <c r="B160" s="35">
+        <v>0.60670000000000002</v>
+      </c>
+      <c r="C160" s="36">
+        <v>2.621E+17</v>
+      </c>
+    </row>
+    <row r="161" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A161" s="35">
+        <v>1075</v>
+      </c>
+      <c r="B161" s="35">
+        <v>0.60609999999999997</v>
+      </c>
+      <c r="C161" s="36">
+        <v>2.638E+17</v>
+      </c>
+    </row>
+    <row r="162" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A162" s="35">
+        <v>1080</v>
+      </c>
+      <c r="B162" s="35">
+        <v>0.59379999999999999</v>
+      </c>
+      <c r="C162" s="36">
+        <v>2.654E+17</v>
+      </c>
+    </row>
+    <row r="163" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A163" s="35">
+        <v>1085</v>
+      </c>
+      <c r="B163" s="35">
+        <v>0.57709999999999995</v>
+      </c>
+      <c r="C163" s="36">
+        <v>2.669E+17</v>
+      </c>
+    </row>
+    <row r="164" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A164" s="35">
+        <v>1090</v>
+      </c>
+      <c r="B164" s="35">
+        <v>0.5756</v>
+      </c>
+      <c r="C164" s="36">
+        <v>2.685E+17</v>
+      </c>
+    </row>
+    <row r="165" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A165" s="35">
+        <v>1095</v>
+      </c>
+      <c r="B165" s="35">
+        <v>0.52890000000000004</v>
+      </c>
+      <c r="C165" s="36">
+        <v>2.7E+17</v>
+      </c>
+    </row>
+    <row r="166" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A166" s="35">
+        <v>1100</v>
+      </c>
+      <c r="B166" s="35">
+        <v>0.49299999999999999</v>
+      </c>
+      <c r="C166" s="36">
+        <v>2.707E+17</v>
+      </c>
+    </row>
+    <row r="167" spans="1:3" ht="16.5" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A167" s="37"/>
+      <c r="B167" s="37"/>
+      <c r="C167" s="37"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A167:C167"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>